<commit_message>
Adicionadas novas funcionalidades : Resgistos Filtros Exportações
</commit_message>
<xml_diff>
--- a/CHECKLIST-ALFA-1/Dados/registos_checklist.xlsx
+++ b/CHECKLIST-ALFA-1/Dados/registos_checklist.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V8"/>
+  <dimension ref="A1:Y12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -497,17 +497,20 @@
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
     <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="8" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
-    <col width="8" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="30" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="8" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="8" customWidth="1" min="24" max="24"/>
+    <col width="30" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -568,55 +571,70 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>Resolução</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Teclado</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Ecrã</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Touch Screen</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Wifi</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>LAN</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Webcam</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Microfone</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Colunas</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>USB</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Portas de Vídeo</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>LTE</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
@@ -670,16 +688,8 @@
           <t>Intel(R) UHD Graphics | NVIDIA GeForce RTX 3070 Laptop GPU</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="3" t="inlineStr">
         <is>
           <t>✓</t>
@@ -705,20 +715,31 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="S2" s="4" t="inlineStr"/>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="U2" s="3" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V2" s="4" t="inlineStr">
-        <is>
-          <t>testes</t>
+      <c r="U2" s="4" t="inlineStr"/>
+      <c r="V2" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W2" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X2" s="4" t="inlineStr"/>
+      <c r="Y2" s="4" t="inlineStr">
+        <is>
+          <t>alterar</t>
         </is>
       </c>
     </row>
@@ -770,16 +791,8 @@
           <t>Intel(R) UHD Graphics | NVIDIA GeForce RTX 3070 Laptop GPU</t>
         </is>
       </c>
-      <c r="L3" s="6" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M3" s="6" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="L3" s="5" t="inlineStr"/>
+      <c r="M3" s="5" t="inlineStr"/>
       <c r="N3" s="6" t="inlineStr">
         <is>
           <t>✓</t>
@@ -805,18 +818,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="S3" s="7" t="inlineStr"/>
+      <c r="S3" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="T3" s="6" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="U3" s="6" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V3" s="7" t="inlineStr">
+      <c r="U3" s="7" t="inlineStr"/>
+      <c r="V3" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W3" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X3" s="7" t="inlineStr"/>
+      <c r="Y3" s="7" t="inlineStr">
         <is>
           <t>Danos para teste</t>
         </is>
@@ -870,16 +894,8 @@
           <t>Intel(R) UHD Graphics | NVIDIA GeForce RTX 3070 Laptop GPU</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="3" t="inlineStr">
         <is>
           <t>✓</t>
@@ -905,18 +921,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="S4" s="4" t="inlineStr"/>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="U4" s="3" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V4" s="4" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr"/>
+      <c r="V4" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W4" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X4" s="4" t="inlineStr"/>
+      <c r="Y4" s="4" t="inlineStr">
         <is>
           <t>teste</t>
         </is>
@@ -974,16 +1001,8 @@
           <t>Intel(R) UHD Graphics | NVIDIA GeForce RTX 3070 Laptop GPU</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M5" s="6" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="L5" s="5" t="inlineStr"/>
+      <c r="M5" s="5" t="inlineStr"/>
       <c r="N5" s="6" t="inlineStr">
         <is>
           <t>✓</t>
@@ -1009,18 +1028,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="S5" s="7" t="inlineStr"/>
+      <c r="S5" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="T5" s="6" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="U5" s="6" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V5" s="7" t="inlineStr">
+      <c r="U5" s="7" t="inlineStr"/>
+      <c r="V5" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W5" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X5" s="7" t="inlineStr"/>
+      <c r="Y5" s="7" t="inlineStr">
         <is>
           <t>teste</t>
         </is>
@@ -1078,16 +1108,8 @@
           <t>NVIDIA GeForce RTX 3070</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M6" s="3" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="3" t="inlineStr">
         <is>
           <t>✓</t>
@@ -1128,7 +1150,18 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V6" s="4" t="inlineStr">
+      <c r="V6" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W6" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X6" s="4" t="inlineStr"/>
+      <c r="Y6" s="4" t="inlineStr">
         <is>
           <t>Sem observações</t>
         </is>
@@ -1186,16 +1219,8 @@
           <t>NVIDIA GeForce RTX 3070</t>
         </is>
       </c>
-      <c r="L7" s="6" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M7" s="6" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="L7" s="5" t="inlineStr"/>
+      <c r="M7" s="5" t="inlineStr"/>
       <c r="N7" s="6" t="inlineStr">
         <is>
           <t>✓</t>
@@ -1236,7 +1261,18 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V7" s="7" t="inlineStr">
+      <c r="V7" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W7" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X7" s="7" t="inlineStr"/>
+      <c r="Y7" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -1298,16 +1334,8 @@
           <t>NVIDIA GeForce RTX 3070</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M8" s="3" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="3" t="inlineStr">
         <is>
           <t>✓</t>
@@ -1348,9 +1376,508 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V8" s="4" t="inlineStr">
+      <c r="V8" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W8" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X8" s="4" t="inlineStr"/>
+      <c r="Y8" s="4" t="inlineStr">
         <is>
           <t>teste alteração</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>24/02/2026 20:49</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Guilherme</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>teste2</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>ASUS System Product Name</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>221011108801049</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>AMD Ryzen 7 5800X3D 8-Core Processor</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>DIMM</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>onboard</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>WD Blue SN570 1TB (932 GB) + Verbatim Vi550 S3 (477 GB)</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 3070</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr"/>
+      <c r="M9" s="5" t="inlineStr"/>
+      <c r="N9" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O9" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P9" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Q9" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R9" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="S9" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T9" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U9" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V9" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W9" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X9" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y9" s="7" t="inlineStr">
+        <is>
+          <t>teste2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>24/02/2026 21:06</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Guilherme</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>ASUS System Product Name</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>221011108801049</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>AMD Ryzen 7 5800X3D 8-Core Processor</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>DIMM</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>WD Blue SN570 1TB (932 GB) + Verbatim Vi550 S3 (477 GB)</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 3070</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>1920x1080</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>239 Hz</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R10" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="S10" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T10" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U10" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V10" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W10" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X10" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y10" s="4" t="inlineStr">
+        <is>
+          <t>teste 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>24/02/2026 21:52</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Guilherme</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>ASUS System Product Name</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>221011108801049</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>AMD Ryzen 7 5800X3D 8-Core Processor</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>DIMM</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr"/>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>WD Blue SN570 1TB (932 GB) + Verbatim Vi550 S3 (477 GB)</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 3070</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>1920x1080</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>144hz</t>
+        </is>
+      </c>
+      <c r="N11" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O11" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P11" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Q11" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R11" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="S11" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T11" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U11" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V11" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W11" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X11" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y11" s="7" t="inlineStr">
+        <is>
+          <t>ddd</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>24/02/2026 22:26</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Guilherme</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>teste1</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>ASUS System Product Name</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>221011108801049</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>AMD Ryzen 7 5800X3D 8-Core Processor</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>DIMM</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>WD Blue SN570 1TB (932 GB) + Verbatim Vi550 S3 (477 GB)</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 3070</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>1920x1080</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>239 Hz</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="S12" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T12" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U12" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V12" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W12" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X12" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y12" s="4" t="inlineStr">
+        <is>
+          <t>teste</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Funcionalidade TVS ADICIONADA na checlist
</commit_message>
<xml_diff>
--- a/CHECKLIST-ALFA-1/Dados/registos_checklist.xlsx
+++ b/CHECKLIST-ALFA-1/Dados/registos_checklist.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y12"/>
+  <dimension ref="A1:Y13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1881,6 +1881,129 @@
         </is>
       </c>
     </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>27/02/2026 20:39</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Guilherme</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>teste</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>ASUS System Product Name</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>221011108801049</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>AMD Ryzen 7 5800X3D 8-Core Processor</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>DIMM</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr"/>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>WD Blue SN570 1TB (932 GB) + Verbatim Vi550 S3 (477 GB)</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 3070</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>1920x1080</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>239 Hz</t>
+        </is>
+      </c>
+      <c r="N13" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O13" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P13" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Q13" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R13" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="S13" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T13" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U13" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V13" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W13" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X13" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y13" s="7" t="inlineStr">
+        <is>
+          <t>pressure marks lcd</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>